<commit_message>
update asakai board, view
</commit_message>
<xml_diff>
--- a/public/template_import_plan.xlsx
+++ b/public/template_import_plan.xlsx
@@ -397,14 +397,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:I3"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -418,12 +421,21 @@
         <v>fgroup</v>
       </c>
       <c r="D1" t="str">
+        <v>ftt</v>
+      </c>
+      <c r="E1" t="str">
+        <v>foee</v>
+      </c>
+      <c r="F1" t="str">
+        <v>fratio</v>
+      </c>
+      <c r="G1" t="str">
         <v>f1tr</v>
       </c>
-      <c r="E1" t="str">
+      <c r="H1" t="str">
         <v>f2tr</v>
       </c>
-      <c r="F1" t="str">
+      <c r="I1" t="str">
         <v>ot</v>
       </c>
     </row>
@@ -438,12 +450,21 @@
         <v>R</v>
       </c>
       <c r="D2">
+        <v>54</v>
+      </c>
+      <c r="E2">
+        <v>95</v>
+      </c>
+      <c r="F2" t="str">
+        <v>60:40</v>
+      </c>
+      <c r="G2">
         <v>120</v>
       </c>
-      <c r="E2">
+      <c r="H2">
         <v>100</v>
       </c>
-      <c r="F2">
+      <c r="I2">
         <v>1.5</v>
       </c>
     </row>
@@ -458,18 +479,27 @@
         <v>W</v>
       </c>
       <c r="D3">
+        <v>54</v>
+      </c>
+      <c r="E3">
+        <v>92</v>
+      </c>
+      <c r="F3" t="str">
+        <v>55:45</v>
+      </c>
+      <c r="G3">
         <v>110</v>
       </c>
-      <c r="E3">
+      <c r="H3">
         <v>95</v>
       </c>
-      <c r="F3">
+      <c r="I3">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update clear daily planning and prod achievement
</commit_message>
<xml_diff>
--- a/public/template_import_plan.xlsx
+++ b/public/template_import_plan.xlsx
@@ -398,17 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I3"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +425,7 @@
         <v>f2tr</v>
       </c>
       <c r="I1" t="str">
-        <v>ot</v>
+        <v>fot</v>
       </c>
     </row>
     <row r="2">

</xml_diff>